<commit_message>
changes to all pys -version 1
</commit_message>
<xml_diff>
--- a/Listings.xlsx
+++ b/Listings.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\PW\Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Science\DSProjects\PWAutomation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F238C389-6A2A-4596-94FA-EA70E5A650D9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CE4B3D-1895-4940-836A-AD035606C893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17256" windowHeight="6636" xr2:uid="{F8867A3C-C405-4EE9-B429-729F4580BC22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F8867A3C-C405-4EE9-B429-729F4580BC22}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>URL</t>
   </si>
@@ -34,16 +34,42 @@
   </si>
   <si>
     <t>https://shopee.sg/Fully-Automatic-Soy-Milk-Maker-Portable-Juicer-Blender-Machine-Smart-Soya-Bean-Milk-Machine-i.299068664.50058759450?extraParams=%7B%22display_model_id%22%3A420778894384%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>https://shopee.sg/%E8%B1%86%E6%B5%86%E6%9C%BA%E5%AE%B6%E7%94%A8%E5%85%A8%E8%87%AA%E5%8A%A8%E5%85%8D%E7%85%AE%E5%85%8D%E6%BB%A4%E9%9D%99%E9%9F%B3%E6%97%A0%E6%B8%A3%E8%BF%B7%E4%BD%A0%E5%A4%9A%E5%8A%9F%E8%83%BD%E6%A6%A8%E6%B1%81%E5%B0%8F%E5%9E%8B%E7%A0%B4%E5%A3%81%E6%9C%BA-i.1257795465.46357553994?extraParams=%7B%22display_model_id%22%3A370671036105%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>https://shopee.sg/%E7%A0%B4%E5%A3%81%E6%9C%BA%E6%A6%A8%E6%B1%81%E6%9C%BA%E4%B8%80%E4%BD%93%E5%AE%B6%E7%94%A8%E9%9D%99%E9%9F%B32025%E5%85%A8%E8%87%AA%E5%8A%A8%E5%B0%8F%E5%9E%8B%E6%97%A0%E6%B8%A3%E5%85%8D%E7%85%AE%E8%B1%86%E6%B5%86%E6%9C%BA-i.1257795465.49057544515?extraParams=%7B%22display_model_id%22%3A345671036006%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>https://shopee.sg/%E5%A4%A7%E5%AE%87%E7%A0%B4%E5%A3%81%E6%9C%BA%E5%AE%B6%E7%94%A8%E5%B0%8F%E5%9E%8B%E8%B1%86%E6%B5%86%E6%9C%BA%E5%85%A8%E8%87%AA%E5%8A%A8%E8%BF%B7%E4%BD%A0%E9%9D%9E%E9%9D%99%E4%BD%8E%E5%99%AA%E9%9F%B3%E6%97%A0%E6%B8%A3%E6%96%B0%E6%AC%BE%E6%A6%A8%E6%B1%81%E7%B1%B3%E7%B3%8ADaewoo-wall-breaking-machine-household-small-soybean-milk-machine-automatic20251127-i.1257795465.53052198783?extraParams=%7B%22display_model_id%22%3A445213452026%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>https://shopee.sg/%E3%80%90BRUNO%E3%80%91Soy-Milk-Maker-Machine-1000ml-High-Speed-Blender-Multifunctional-Food-Processor-High-borosilicate-Glass-Liner-i.1343862364.54707001967?extraParams=%7B%22display_model_id%22%3A208812747787%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>https://shopee.sg/%E3%80%90BRUNO%E3%80%91Soy-Milk-Maker-Machine-Blender-Milk-Pot-Jug-Soya-Bean-Machine-600-1000ml-316-Stainless-Steel-i.1343862364.44129362157?extraParams=%7B%22display_model_id%22%3A345658530595%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>https://shopee.sg/NEW-Mini-soymilk-maker-1600ml-blender-heating-blender-Multifunctional-wall-breaker-48-blades-i.1457582756.56909241870?extraParams=%7B%22display_model_id%22%3A350817897757%2C%22model_selection_logic%22%3A3%7D</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -66,13 +92,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -385,7 +414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7BC95AD-EF11-4653-9716-E76E6BC2B239}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -403,8 +432,43 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A7" r:id="rId1" display="https://shopee.sg/%E3%80%90BRUNO%E3%80%91Soy-Milk-Maker-Machine-1000ml-High-Speed-Blender-Multifunctional-Food-Processor-High-borosilicate-Glass-Liner-i.1343862364.54707001967?extraParams=%7B%22display_model_id%22%3A208812747787%2C%22model_selection_logic%22%3A3%7D" xr:uid="{1E158D23-BE59-491A-9071-CFB6B4F05A77}"/>
+    <hyperlink ref="A8" r:id="rId2" xr:uid="{DFC22605-9D45-48CB-941F-B063F37178EB}"/>
+    <hyperlink ref="A9" r:id="rId3" xr:uid="{DAD3C609-B024-4DD8-B628-D3D11FFD044C}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>